<commit_message>
Update selector to match groups without `field-list`
</commit_message>
<xml_diff>
--- a/tests/e2e/default/enketo/forms/db-object-form.xlsx
+++ b/tests/e2e/default/enketo/forms/db-object-form.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="survey" sheetId="1" state="visible" r:id="rId3"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="42">
   <si>
     <t xml:space="preserve">type</t>
   </si>
@@ -62,33 +62,36 @@
     <t xml:space="preserve">contact_id</t>
   </si>
   <si>
+    <t xml:space="preserve">select-contact type-person</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hidden</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sex</t>
+  </si>
+  <si>
+    <t xml:space="preserve">end_group</t>
+  </si>
+  <si>
+    <t xml:space="preserve">user_contact</t>
+  </si>
+  <si>
+    <t xml:space="preserve">_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">../../inputs/user/contact_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">people</t>
+  </si>
+  <si>
+    <t xml:space="preserve">field-list</t>
+  </si>
+  <si>
     <t xml:space="preserve">hidden select-contact type-person</t>
   </si>
   <si>
-    <t xml:space="preserve">hidden</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sex</t>
-  </si>
-  <si>
-    <t xml:space="preserve">end_group</t>
-  </si>
-  <si>
-    <t xml:space="preserve">user_contact</t>
-  </si>
-  <si>
-    <t xml:space="preserve">_id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">../../user/contact_id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">people</t>
-  </si>
-  <si>
-    <t xml:space="preserve">field-list</t>
-  </si>
-  <si>
     <t xml:space="preserve">../../../inputs/user/contact_id</t>
   </si>
   <si>
@@ -105,9 +108,6 @@
   </si>
   <si>
     <t xml:space="preserve">Select a person from all</t>
-  </si>
-  <si>
-    <t xml:space="preserve">select-contact type-person</t>
   </si>
   <si>
     <t xml:space="preserve">title</t>
@@ -249,16 +249,12 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -314,37 +310,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="44546a"/>
+        <a:srgbClr val="44546A"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="e7e6e6"/>
+        <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4472c4"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ed7d31"/>
+        <a:srgbClr val="ED7D31"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a5a5a5"/>
+        <a:srgbClr val="A5A5A5"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="ffc000"/>
+        <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="5b9bd5"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="70ad47"/>
+        <a:srgbClr val="70AD47"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0563c1"/>
+        <a:srgbClr val="0563C1"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="954f72"/>
+        <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -483,8 +479,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:XFB1048576"/>
-  <sheetFormatPr defaultColWidth="14.66796875" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:G1048576"/>
+  <sheetFormatPr defaultColWidth="14.66796875" defaultRowHeight="12.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.53"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="21.98"/>
@@ -495,388 +491,366 @@
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1010" min="7" style="1" width="14.67"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1015" min="1011" style="1" width="11.5"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16378" min="1016" style="1" width="14.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16379" min="16379" style="2" width="11.53"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16382" min="16380" style="1" width="11.53"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16383" style="2" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16379" style="1" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="4"/>
+      <c r="G1" s="3"/>
     </row>
     <row r="2" customFormat="false" ht="15.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" s="6"/>
-      <c r="E2" s="5" t="s">
+      <c r="C2" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="4"/>
+      <c r="E2" s="1" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="5"/>
-      <c r="B3" s="5"/>
-      <c r="C3" s="5"/>
-      <c r="D3" s="6"/>
-      <c r="E3" s="5"/>
+      <c r="A3" s="4"/>
+      <c r="B3" s="4"/>
+      <c r="C3" s="4"/>
+      <c r="D3" s="5"/>
+      <c r="E3" s="4"/>
     </row>
     <row r="4" customFormat="false" ht="15.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D4" s="6"/>
-      <c r="E4" s="5"/>
+      <c r="C4" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" s="5"/>
+      <c r="E4" s="4"/>
     </row>
     <row r="5" customFormat="false" ht="15.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D5" s="6" t="s">
+      <c r="C5" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D5" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E5" s="5"/>
+      <c r="E5" s="4"/>
     </row>
     <row r="6" customFormat="false" ht="15.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D6" s="6"/>
-      <c r="E6" s="5"/>
+      <c r="C6" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D6" s="5"/>
+      <c r="E6" s="4"/>
     </row>
     <row r="7" customFormat="false" ht="15.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C7" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D7" s="6"/>
-      <c r="E7" s="5"/>
+      <c r="C7" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D7" s="5"/>
+      <c r="E7" s="4"/>
     </row>
     <row r="8" customFormat="false" ht="15.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="5"/>
-      <c r="D8" s="6"/>
-      <c r="E8" s="5"/>
+      <c r="C8" s="4"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="4"/>
     </row>
     <row r="9" customFormat="false" ht="15.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5"/>
-      <c r="B9" s="5"/>
-      <c r="C9" s="5"/>
-      <c r="D9" s="6"/>
-      <c r="E9" s="5"/>
+      <c r="A9" s="4"/>
+      <c r="B9" s="4"/>
+      <c r="C9" s="4"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="4"/>
     </row>
     <row r="10" customFormat="false" ht="15.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5" t="s">
+      <c r="A10" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10" s="4"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="4"/>
+    </row>
+    <row r="11" customFormat="false" ht="15.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4"/>
+      <c r="B11" s="4"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="5"/>
+      <c r="E11" s="4"/>
+    </row>
+    <row r="12" customFormat="false" ht="15.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B12" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D10" s="6"/>
-      <c r="E10" s="5"/>
-    </row>
-    <row r="11" customFormat="false" ht="15.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="5" t="s">
+      <c r="C12" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B13" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D11" s="6" t="s">
+      <c r="C13" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D13" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E11" s="5"/>
-      <c r="F11" s="1" t="s">
+      <c r="E13" s="4"/>
+      <c r="F13" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="5" t="s">
+    <row r="14" customFormat="false" ht="15.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B14" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C12" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D12" s="6"/>
-      <c r="E12" s="5"/>
-    </row>
-    <row r="13" customFormat="false" ht="15.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5" t="s">
+      <c r="C14" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D14" s="5"/>
+      <c r="E14" s="4"/>
+    </row>
+    <row r="15" customFormat="false" ht="15.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B15" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C13" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D13" s="6"/>
-      <c r="E13" s="5"/>
-    </row>
-    <row r="14" customFormat="false" ht="15.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="5" t="s">
+      <c r="C15" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D15" s="5"/>
+      <c r="E15" s="4"/>
+    </row>
+    <row r="16" customFormat="false" ht="15.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B16" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C14" s="5"/>
-      <c r="D14" s="6"/>
-      <c r="E14" s="5"/>
-    </row>
-    <row r="15" customFormat="false" ht="15.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="5"/>
-      <c r="B15" s="5"/>
-      <c r="C15" s="5"/>
-      <c r="D15" s="6"/>
-      <c r="E15" s="5"/>
-    </row>
-    <row r="16" customFormat="false" ht="15.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="5" t="s">
+      <c r="C16" s="4"/>
+      <c r="D16" s="5"/>
+      <c r="E16" s="4"/>
+    </row>
+    <row r="17" customFormat="false" ht="15.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4"/>
+      <c r="B17" s="4"/>
+      <c r="C17" s="4"/>
+      <c r="D17" s="5"/>
+      <c r="E17" s="4"/>
+    </row>
+    <row r="18" customFormat="false" ht="15.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="E18" s="4"/>
+    </row>
+    <row r="19" customFormat="false" ht="15.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="6"/>
+      <c r="B19" s="6"/>
+      <c r="C19" s="6"/>
+      <c r="D19" s="7"/>
+      <c r="E19" s="4"/>
+    </row>
+    <row r="20" customFormat="false" ht="15.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D20" s="5"/>
+      <c r="E20" s="4"/>
+    </row>
+    <row r="21" customFormat="false" ht="15.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E21" s="4"/>
+      <c r="F21" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D22" s="5"/>
+      <c r="E22" s="4"/>
+    </row>
+    <row r="23" customFormat="false" ht="15.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D23" s="5"/>
+      <c r="E23" s="4"/>
+    </row>
+    <row r="24" customFormat="false" ht="15.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B16" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C16" s="5"/>
-      <c r="D16" s="6"/>
-      <c r="E16" s="5"/>
-    </row>
-    <row r="17" customFormat="false" ht="15.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="5"/>
-      <c r="B17" s="5"/>
-      <c r="C17" s="5"/>
-      <c r="D17" s="6"/>
-      <c r="E17" s="5"/>
-    </row>
-    <row r="18" customFormat="false" ht="15.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="5"/>
-      <c r="B18" s="5"/>
-      <c r="C18" s="5"/>
-      <c r="D18" s="6"/>
-      <c r="E18" s="5"/>
-    </row>
-    <row r="19" customFormat="false" ht="15.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="B19" s="7" t="s">
+      <c r="B24" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C24" s="4"/>
+      <c r="D24" s="5"/>
+      <c r="E24" s="4"/>
+    </row>
+    <row r="25" customFormat="false" ht="15.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="6"/>
+      <c r="B25" s="6"/>
+      <c r="C25" s="6"/>
+      <c r="D25" s="7"/>
+      <c r="E25" s="4"/>
+    </row>
+    <row r="26" customFormat="false" ht="15.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D26" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="E26" s="4"/>
+    </row>
+    <row r="27" customFormat="false" ht="15.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="D27" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E27" s="4"/>
+    </row>
+    <row r="28" customFormat="false" ht="15.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="4"/>
+      <c r="B28" s="4"/>
+      <c r="C28" s="4"/>
+      <c r="D28" s="5"/>
+      <c r="E28" s="4"/>
+    </row>
+    <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B29" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="C19" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="D19" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="E19" s="5"/>
-    </row>
-    <row r="20" customFormat="false" ht="15.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="7"/>
-      <c r="B20" s="7"/>
-      <c r="C20" s="7"/>
-      <c r="D20" s="8"/>
-      <c r="E20" s="5"/>
-    </row>
-    <row r="21" customFormat="false" ht="15.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B21" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="C21" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D21" s="6"/>
-      <c r="E21" s="5"/>
-      <c r="XEZ21" s="2"/>
-      <c r="XFA21" s="2"/>
-      <c r="XFB21" s="2"/>
-    </row>
-    <row r="22" customFormat="false" ht="15.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="B22" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="C22" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D22" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="E22" s="5"/>
-      <c r="F22" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="XEZ22" s="2"/>
-      <c r="XFA22" s="2"/>
-      <c r="XFB22" s="2"/>
-    </row>
-    <row r="23" customFormat="false" ht="15.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B23" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="C23" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D23" s="6"/>
-      <c r="E23" s="5"/>
-      <c r="XEZ23" s="2"/>
-      <c r="XFA23" s="2"/>
-      <c r="XFB23" s="2"/>
-    </row>
-    <row r="24" customFormat="false" ht="15.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B24" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C24" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D24" s="6"/>
-      <c r="E24" s="5"/>
-      <c r="XEZ24" s="2"/>
-      <c r="XFA24" s="2"/>
-      <c r="XFB24" s="2"/>
-    </row>
-    <row r="25" customFormat="false" ht="15.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B25" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="C25" s="5"/>
-      <c r="D25" s="6"/>
-      <c r="E25" s="5"/>
-      <c r="XEZ25" s="2"/>
-      <c r="XFA25" s="2"/>
-      <c r="XFB25" s="2"/>
-    </row>
-    <row r="26" customFormat="false" ht="15.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="7"/>
-      <c r="B26" s="7"/>
-      <c r="C26" s="7"/>
-      <c r="D26" s="8"/>
-      <c r="E26" s="5"/>
-    </row>
-    <row r="27" customFormat="false" ht="15.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="B27" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="C27" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="D27" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="E27" s="5"/>
-    </row>
-    <row r="28" customFormat="false" ht="15.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="B28" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="C28" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="D28" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="E28" s="5"/>
-    </row>
-    <row r="29" customFormat="false" ht="15.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="5"/>
-      <c r="B29" s="5"/>
       <c r="C29" s="5"/>
-      <c r="D29" s="6"/>
+      <c r="D29" s="5"/>
       <c r="E29" s="5"/>
-    </row>
-    <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="B30" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="C30" s="6"/>
-      <c r="D30" s="6"/>
-      <c r="E30" s="6"/>
-      <c r="F30" s="6"/>
-      <c r="G30" s="6"/>
-    </row>
+      <c r="F29" s="5"/>
+      <c r="G29" s="5"/>
+    </row>
+    <row r="1048559" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048560" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048561" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048562" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -911,7 +885,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G2"/>
-  <sheetFormatPr defaultColWidth="14.66796875" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.66796875" defaultRowHeight="12.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="1" style="1" width="17.33"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="18.16"/>
@@ -920,38 +894,38 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="2" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="8" t="s">
+      <c r="A2" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="C2" s="9" t="n">
+      <c r="C2" s="8" t="n">
         <f aca="true">TODAY()</f>
-        <v>45540</v>
+        <v>46142</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>38</v>
@@ -962,7 +936,7 @@
       <c r="F2" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="G2" s="10" t="s">
+      <c r="G2" s="9" t="s">
         <v>41</v>
       </c>
     </row>

</xml_diff>